<commit_message>
feat: Enhance inspiration board functionality and performance
- Added `created` property to `FabricaUser` type for tracking user creation time.
- Improved circle hit testing algorithm in `canvasElementAt` function for better accuracy.
- Implemented edit functionality for inspiration items in the inspiration browser test.
- Introduced `InspirationCanvas` component for rendering canvas elements with optimized drawing logic.
- Created `inspiration-scene` module for managing canvas elements, including spatial indexing and stroke simplification.
- Added comprehensive tests for the new functionality, including validation of canvas elements and performance benchmarks for spatial queries.
</commit_message>
<xml_diff>
--- a/outputs/outreach-sept-2026/prospectos-fabrica-septiembre-2026.xlsx
+++ b/outputs/outreach-sept-2026/prospectos-fabrica-septiembre-2026.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospectos" sheetId="1" r:id="R0ef59e9f06554b42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospectos" sheetId="1" r:id="Ra974073456e74fa1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -151,7 +151,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="37">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -242,6 +242,7 @@
     <x:xf numFmtId="200" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -253,7 +254,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -264,7 +265,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -274,7 +275,7 @@
         <x:color rgb="FF075985"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE0F2FE"/>
         </x:patternFill>
       </x:fill>
@@ -284,7 +285,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProspectosTable" displayName="ProspectosTable" ref="A7:F67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProspectosTable" displayName="ProspectosTable" ref="A7:F98" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Estudio / contacto"/>
     <x:tableColumn id="2" name="Email"/>
@@ -530,8 +531,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="12" t="n">
-        <x:f>COUNTA(A8:A67)</x:f>
-        <x:v>60</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B5" s="12" t="n">
         <x:f>COUNTIF(E8:E67,"Caliente")</x:f>
@@ -1647,6 +1647,588 @@
         <x:v>Contactado</x:v>
       </x:c>
       <x:c r="F67" s="34" t="str"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>Primer Piso Arquitectos</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>info.primerpisoarquitectos@gmail.com</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>Arquitectura</x:v>
+      </x:c>
+      <x:c r="D68" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E68" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F68"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
+        <x:v>Before &amp; After</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>arquitectura@beforeandafter.com.ar</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>Arquitectura</x:v>
+      </x:c>
+      <x:c r="D69" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E69" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F69"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>MJV Estudio — María José Varas</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>jochivaras@gmail.com</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>Arquitectura e interiores</x:v>
+      </x:c>
+      <x:c r="D70" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F70"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>Andia Andia</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>andiaarquing@gmail.com</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>Arquitectura e ingeniería</x:v>
+      </x:c>
+      <x:c r="D71" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F71"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>In Estudio Arquitectura — Daniel Gelardi</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>danielgelardi@gmail.com</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>Arquitectura</x:v>
+      </x:c>
+      <x:c r="D72" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F72"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>In Estudio Arquitectura — Federico Inchauspe</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>federicoinchauspe@gmail.com</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>Arquitectura</x:v>
+      </x:c>
+      <x:c r="D73" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F73"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>Tresde Studio</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>tresde.studiomza@gmail.com</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>Arquitectura</x:v>
+      </x:c>
+      <x:c r="D74" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F74"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>Sustent Arq</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>sustentaarq@gmail.com</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>Arquitectura</x:v>
+      </x:c>
+      <x:c r="D75" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F75"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>Rosana Raffaini Arquitectura</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>arquitectaraffaini@gmail.com</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>Arquitectura</x:v>
+      </x:c>
+      <x:c r="D76" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F76"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>Astoria Construcciones Civiles</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>administracion@astoriacc.com.ar</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>Ingeniería civil</x:v>
+      </x:c>
+      <x:c r="D77" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F77"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>Ingeniería M.EM.G</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>direccion@ingenieriamemg.com</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>Ingeniería civil</x:v>
+      </x:c>
+      <x:c r="D78" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E78" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F78"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>Constructora San Guillermo</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>contacto@constructorasanguillermo.com.ar</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>Ingeniería civil</x:v>
+      </x:c>
+      <x:c r="D79" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F79"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>KIRIOS Ingeniería y Construcción</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>info@kiriossa.com.ar</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>Ingeniería civil</x:v>
+      </x:c>
+      <x:c r="D80" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F80"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>Noelia Reveco Ingeniería</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>nreveco.ing@gmail.com</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>Ingeniería civil</x:v>
+      </x:c>
+      <x:c r="D81" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F81"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>Hinrichsen Industrial Design Studio</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>enzohinrichsen@gmail.com</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>Diseño industrial</x:v>
+      </x:c>
+      <x:c r="D82" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F82"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="str">
+        <x:v>MYT Soluciones</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>hola@mytsoluciones.com</x:v>
+      </x:c>
+      <x:c r="C83" t="str">
+        <x:v>Diseño industrial</x:v>
+      </x:c>
+      <x:c r="D83" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E83" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F83"/>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>TEC3D</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>cotizaciones@tec3d.com.ar</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>Diseño industrial</x:v>
+      </x:c>
+      <x:c r="D84" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E84" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F84"/>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="str">
+        <x:v>Walter Galesi Interiorismo</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>waltergalesi.interiorismo@gmail.com</x:v>
+      </x:c>
+      <x:c r="C85" t="str">
+        <x:v>Diseño de interiores</x:v>
+      </x:c>
+      <x:c r="D85" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E85" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F85"/>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>Naranjo Interiorismo</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>info@naranjotiendaonline.com.ar</x:v>
+      </x:c>
+      <x:c r="C86" t="str">
+        <x:v>Diseño de interiores</x:v>
+      </x:c>
+      <x:c r="D86" s="36" t="n">
+        <x:v>46283.625</x:v>
+      </x:c>
+      <x:c r="E86" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F86"/>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>Renders Studio</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>renders.studio3d@gmail.com</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>Renderizado 3D</x:v>
+      </x:c>
+      <x:c r="D87" s="36" t="n">
+        <x:v>46286.625</x:v>
+      </x:c>
+      <x:c r="E87" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F87" t="str">
+        <x:v>Demo adjunta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="str">
+        <x:v>Jorge Peralta</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>info3d.jorge@gmail.com</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>Renderizado 3D</x:v>
+      </x:c>
+      <x:c r="D88" s="36" t="n">
+        <x:v>46286.625</x:v>
+      </x:c>
+      <x:c r="E88" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F88" t="str">
+        <x:v>Demo adjunta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="str">
+        <x:v>Estudio Mendoza — Guido Elgueta</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>ge@estudiomendoza.com</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>Visualización arquitectónica 3D</x:v>
+      </x:c>
+      <x:c r="D89" s="36" t="n">
+        <x:v>46286.625</x:v>
+      </x:c>
+      <x:c r="E89" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F89" t="str">
+        <x:v>Demo adjunta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="str">
+        <x:v>Estudio Mendoza — Marcos Elgueta</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>me@estudiomendoza.com</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>Visualización arquitectónica 3D</x:v>
+      </x:c>
+      <x:c r="D90" s="36" t="n">
+        <x:v>46286.625</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F90" t="str">
+        <x:v>Demo adjunta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>González Olsina &amp; Vega</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>gestionintegracpm@gmail.com</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>Arquitectura</x:v>
+      </x:c>
+      <x:c r="D91" s="36" t="n">
+        <x:v>46286.625</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F91" t="str">
+        <x:v>Demo adjunta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>KUBO Arquitectura</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>s.baigorria@kuboarq.com.ar</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>Arquitectura</x:v>
+      </x:c>
+      <x:c r="D92" s="36" t="n">
+        <x:v>46286.625</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F92" t="str">
+        <x:v>Demo adjunta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>A4estudio</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>info@a4estudio.com.ar</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>Arquitectura</x:v>
+      </x:c>
+      <x:c r="D93" s="36" t="n">
+        <x:v>46286.625</x:v>
+      </x:c>
+      <x:c r="E93" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F93" t="str">
+        <x:v>Demo adjunta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>G Studio Render</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>g.studiorender@gmail.com</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>Renderizado 3D</x:v>
+      </x:c>
+      <x:c r="D94" s="36" t="n">
+        <x:v>46286.625</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F94" t="str">
+        <x:v>Demo adjunta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>YGC Arquitectos</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>info@yancarelligomez.com.ar</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>Arquitectura e interiores</x:v>
+      </x:c>
+      <x:c r="D95" s="36" t="n">
+        <x:v>46286.625</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F95" t="str">
+        <x:v>Demo adjunta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>We Design</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>somos.wedesign@gmail.com</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>Arquitectura y visualización 3D</x:v>
+      </x:c>
+      <x:c r="D96" s="36" t="n">
+        <x:v>46286.625</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F96" t="str">
+        <x:v>Demo adjunta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>Fukuoka Studio</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>fukuokadis@gmail.com</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>Visualización arquitectónica 3D</x:v>
+      </x:c>
+      <x:c r="D97" s="36" t="n">
+        <x:v>46286.625</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Demo adjunta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>STAV ARQ</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>stav.arq3dbf86cf1e-4a1a-4c06-bdf7-9e2bcef9250b@gmail.com</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>Visualización arquitectónica 3D</x:v>
+      </x:c>
+      <x:c r="D98" s="36" t="n">
+        <x:v>46286.625</x:v>
+      </x:c>
+      <x:c r="E98" t="str">
+        <x:v>Contactado</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>Demo adjunta</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1660,7 +2242,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19d7d5c37ad745c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ed7a3423a7e4281"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>